<commit_message>
modified:   README.md 	new file:   __pycache__/new.cpython-313.pyc 	modified:   __pycache__/use_model.cpython-313.pyc 	modified:   new.py 	modified:   outputs/model_config.json 	modified:   outputs/model_data.h 	modified:   outputs/scaler_x.pkl 	modified:   outputs/scaler_y.pkl 	modified:   outputs/training_log.txt 	modified:   outputs/water_quality_model.pth 	modified:   shuizhi.xlsx 	modified:   "\347\245\236\347\273\217\347\275\221\347\273\234\350\256\255\347\273\203\350\257\264\346\230\216.md"
</commit_message>
<xml_diff>
--- a/shuizhi.xlsx
+++ b/shuizhi.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\STM32\Water_2\Water_Python\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\STM32\Water_Python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9291B1E-C659-4EA5-ADD3-C1B79C1AB918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AAFAC04-A0D3-4087-9575-D825F782CBCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10220" yWindow="1990" windowWidth="19010" windowHeight="9570" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,16 +27,13 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
+    <t>tem</t>
+  </si>
+  <si>
     <t>cod</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>uv254</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>tem</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -361,7 +358,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -372,863 +369,812 @@
         <v>550</v>
       </c>
       <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s">
         <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" t="s">
-        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>0.35884300000000002</v>
+        <v>-0.66940599999999995</v>
       </c>
       <c r="B2">
-        <v>0.54744199999999998</v>
+        <v>0.99091700000000005</v>
       </c>
       <c r="C2">
-        <v>26.912500000000001</v>
+        <v>34.924999999999997</v>
       </c>
       <c r="D2">
-        <v>2.5099999999999998</v>
+        <v>9.32</v>
       </c>
       <c r="E2">
-        <v>6.5000000000000002E-2</v>
+        <v>0.24540000000000001</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>0.35884300000000002</v>
+        <v>-0.67147000000000001</v>
       </c>
       <c r="B3">
-        <v>0.54814399999999996</v>
+        <v>0.98464700000000005</v>
       </c>
       <c r="C3">
-        <v>27.0063</v>
+        <v>35.612499999999997</v>
       </c>
       <c r="D3">
-        <v>2.6</v>
+        <v>9.32</v>
       </c>
       <c r="E3">
-        <v>6.7400000000000002E-2</v>
+        <v>0.24540000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>0.35675600000000002</v>
+        <v>-0.66614399999999996</v>
       </c>
       <c r="B4">
-        <v>0.54961700000000002</v>
+        <v>0.99014899999999995</v>
       </c>
       <c r="C4">
-        <v>27.1187</v>
+        <v>35.524999999999999</v>
       </c>
       <c r="D4">
-        <v>2.57</v>
+        <v>9.32</v>
       </c>
       <c r="E4">
-        <v>6.6600000000000006E-2</v>
+        <v>0.24540000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>0.35509800000000002</v>
+        <v>-0.66018100000000002</v>
       </c>
       <c r="B5">
-        <v>0.54981100000000005</v>
+        <v>0.98134500000000002</v>
       </c>
       <c r="C5">
-        <v>27.237500000000001</v>
+        <v>35.462499999999999</v>
       </c>
       <c r="D5">
-        <v>2.54</v>
+        <v>9.32</v>
       </c>
       <c r="E5">
-        <v>6.5799999999999997E-2</v>
+        <v>0.24540000000000001</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>0.35614200000000001</v>
+        <v>-0.66929000000000005</v>
       </c>
       <c r="B6">
-        <v>0.54699200000000003</v>
+        <v>0.98554900000000001</v>
       </c>
       <c r="C6">
-        <v>27.337499999999999</v>
+        <v>35.4</v>
       </c>
       <c r="D6">
-        <v>2.54</v>
+        <v>9.32</v>
       </c>
       <c r="E6">
-        <v>6.5799999999999997E-2</v>
+        <v>0.24540000000000001</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>0.34610299999999999</v>
+        <v>-0.66615800000000003</v>
       </c>
       <c r="B7">
-        <v>0.54958899999999999</v>
+        <v>0.98964200000000002</v>
       </c>
       <c r="C7">
-        <v>28.281300000000002</v>
+        <v>35.262500000000003</v>
       </c>
       <c r="D7">
-        <v>3.53</v>
+        <v>9.32</v>
       </c>
       <c r="E7">
-        <v>9.1800000000000007E-2</v>
+        <v>0.24540000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>0.345827</v>
+        <v>-0.73696899999999999</v>
       </c>
       <c r="B8">
-        <v>0.54967999999999995</v>
+        <v>0.98286899999999999</v>
       </c>
       <c r="C8">
-        <v>28.35</v>
+        <v>34.15</v>
       </c>
       <c r="D8">
-        <v>3.59</v>
+        <v>3.49</v>
       </c>
       <c r="E8">
-        <v>9.3600000000000003E-2</v>
+        <v>9.0999999999999998E-2</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>0.34530499999999997</v>
+        <v>-0.74681600000000004</v>
       </c>
       <c r="B9">
-        <v>0.54986500000000005</v>
+        <v>0.98243499999999995</v>
       </c>
       <c r="C9">
-        <v>28.4438</v>
+        <v>34.125</v>
       </c>
       <c r="D9">
-        <v>3.56</v>
+        <v>3.49</v>
       </c>
       <c r="E9">
-        <v>9.2700000000000005E-2</v>
+        <v>9.0999999999999998E-2</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>0.34426099999999998</v>
+        <v>-0.75266100000000002</v>
       </c>
       <c r="B10">
-        <v>0.55132300000000001</v>
+        <v>0.98913600000000002</v>
       </c>
       <c r="C10">
-        <v>28.537500000000001</v>
+        <v>34.087499999999999</v>
       </c>
       <c r="D10">
-        <v>3.56</v>
+        <v>3.49</v>
       </c>
       <c r="E10">
-        <v>9.2700000000000005E-2</v>
+        <v>9.0999999999999998E-2</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>0.34601100000000001</v>
+        <v>-0.73510600000000004</v>
       </c>
       <c r="B11">
-        <v>0.55150600000000005</v>
+        <v>0.98113899999999998</v>
       </c>
       <c r="C11">
-        <v>28.5063</v>
+        <v>34.0625</v>
       </c>
       <c r="D11">
-        <v>3.53</v>
+        <v>3.49</v>
       </c>
       <c r="E11">
-        <v>9.1800000000000007E-2</v>
+        <v>9.0999999999999998E-2</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>0.35497499999999998</v>
+        <v>-0.73441199999999995</v>
       </c>
       <c r="B12">
-        <v>0.55775699999999995</v>
+        <v>0.98439399999999999</v>
       </c>
       <c r="C12">
-        <v>37.2562</v>
+        <v>34.0625</v>
       </c>
       <c r="D12">
-        <v>4.38</v>
+        <v>3.49</v>
       </c>
       <c r="E12">
-        <v>0.1145</v>
+        <v>9.0999999999999998E-2</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>0.35537400000000002</v>
+        <v>-0.732352</v>
       </c>
       <c r="B13">
-        <v>0.55674999999999997</v>
+        <v>0.98550899999999997</v>
       </c>
       <c r="C13">
-        <v>37.412500000000001</v>
+        <v>34.0625</v>
       </c>
       <c r="D13">
-        <v>4.49</v>
+        <v>3.49</v>
       </c>
       <c r="E13">
-        <v>0.1174</v>
+        <v>9.0999999999999998E-2</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>0.35571199999999997</v>
+        <v>-0.59872700000000001</v>
       </c>
       <c r="B14">
-        <v>0.55715099999999995</v>
+        <v>0.98803600000000003</v>
       </c>
       <c r="C14">
-        <v>37.518700000000003</v>
+        <v>33.774999999999999</v>
       </c>
       <c r="D14">
-        <v>4.45</v>
+        <v>11.23</v>
       </c>
       <c r="E14">
-        <v>0.1164</v>
+        <v>0.29609999999999997</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>0.35540500000000003</v>
+        <v>-0.59635000000000005</v>
       </c>
       <c r="B15">
-        <v>0.55763399999999996</v>
+        <v>0.98769099999999999</v>
       </c>
       <c r="C15">
-        <v>37.6188</v>
+        <v>33.774999999999999</v>
       </c>
       <c r="D15">
-        <v>4.3099999999999996</v>
+        <v>11.23</v>
       </c>
       <c r="E15">
-        <v>0.11269999999999999</v>
+        <v>0.29609999999999997</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>0.35644900000000002</v>
+        <v>-0.60497999999999996</v>
       </c>
       <c r="B16">
-        <v>0.55790300000000004</v>
+        <v>0.98222900000000002</v>
       </c>
       <c r="C16">
-        <v>37.706200000000003</v>
+        <v>33.75</v>
       </c>
       <c r="D16">
-        <v>4.3099999999999996</v>
+        <v>11.23</v>
       </c>
       <c r="E16">
-        <v>0.11269999999999999</v>
+        <v>0.29609999999999997</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>0.33621800000000002</v>
+        <v>-0.59446600000000005</v>
       </c>
       <c r="B17">
-        <v>0.55282500000000001</v>
+        <v>0.98323099999999997</v>
       </c>
       <c r="C17">
-        <v>31.843800000000002</v>
+        <v>33.75</v>
       </c>
       <c r="D17">
-        <v>3.14</v>
+        <v>11.23</v>
       </c>
       <c r="E17">
-        <v>8.1500000000000003E-2</v>
+        <v>0.29609999999999997</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>0.33514300000000002</v>
+        <v>-0.59125099999999997</v>
       </c>
       <c r="B18">
-        <v>0.55378499999999997</v>
+        <v>0.98957700000000004</v>
       </c>
       <c r="C18">
-        <v>31.968800000000002</v>
+        <v>33.787500000000001</v>
       </c>
       <c r="D18">
-        <v>3.17</v>
+        <v>11.23</v>
       </c>
       <c r="E18">
-        <v>8.2299999999999998E-2</v>
+        <v>0.29609999999999997</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>0.33686300000000002</v>
+        <v>-0.64357600000000004</v>
       </c>
       <c r="B19">
-        <v>0.55351399999999995</v>
+        <v>0.97965000000000002</v>
       </c>
       <c r="C19">
-        <v>31.975000000000001</v>
+        <v>33.787500000000001</v>
       </c>
       <c r="D19">
-        <v>3.14</v>
+        <v>6.51</v>
       </c>
       <c r="E19">
-        <v>8.1500000000000003E-2</v>
+        <v>0.17100000000000001</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>0.33615699999999998</v>
+        <v>-0.66238799999999998</v>
       </c>
       <c r="B20">
-        <v>0.55380700000000005</v>
+        <v>0.98228499999999996</v>
       </c>
       <c r="C20">
-        <v>31.968800000000002</v>
+        <v>33.774999999999999</v>
       </c>
       <c r="D20">
-        <v>3.17</v>
+        <v>6.51</v>
       </c>
       <c r="E20">
-        <v>8.2299999999999998E-2</v>
+        <v>0.17100000000000001</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>0.33382299999999998</v>
+        <v>-0.65145699999999995</v>
       </c>
       <c r="B21">
-        <v>0.55400499999999997</v>
+        <v>0.98225499999999999</v>
       </c>
       <c r="C21">
-        <v>31.843800000000002</v>
+        <v>33.787500000000001</v>
       </c>
       <c r="D21">
-        <v>3.07</v>
+        <v>6.51</v>
       </c>
       <c r="E21">
-        <v>7.9799999999999996E-2</v>
+        <v>0.17100000000000001</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>0.32685500000000001</v>
+        <v>-0.64771500000000004</v>
       </c>
       <c r="B22">
-        <v>0.55223699999999998</v>
+        <v>0.98693500000000001</v>
       </c>
       <c r="C22">
-        <v>30.162500000000001</v>
+        <v>33.774999999999999</v>
       </c>
       <c r="D22">
-        <v>2.82</v>
+        <v>6.51</v>
       </c>
       <c r="E22">
-        <v>7.3099999999999998E-2</v>
+        <v>0.17100000000000001</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>0.32955600000000002</v>
+        <v>-0.65688000000000002</v>
       </c>
       <c r="B23">
-        <v>0.55204399999999998</v>
+        <v>0.98248000000000002</v>
       </c>
       <c r="C23">
-        <v>30.024999999999999</v>
+        <v>33.787500000000001</v>
       </c>
       <c r="D23">
-        <v>2.79</v>
+        <v>6.51</v>
       </c>
       <c r="E23">
-        <v>7.2300000000000003E-2</v>
+        <v>0.17100000000000001</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>0.33170500000000003</v>
+        <v>-0.65862600000000004</v>
       </c>
       <c r="B24">
-        <v>0.55223100000000003</v>
+        <v>0.98651100000000003</v>
       </c>
       <c r="C24">
-        <v>29.8188</v>
+        <v>33.8125</v>
       </c>
       <c r="D24">
-        <v>2.76</v>
+        <v>6.51</v>
       </c>
       <c r="E24">
-        <v>7.1499999999999994E-2</v>
+        <v>0.17100000000000001</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>0.33471400000000001</v>
+        <v>-0.58247199999999999</v>
       </c>
       <c r="B25">
-        <v>0.55167500000000003</v>
+        <v>0.98438499999999995</v>
       </c>
       <c r="C25">
-        <v>29.55</v>
+        <v>33.8125</v>
       </c>
       <c r="D25">
-        <v>2.73</v>
+        <v>10.92</v>
       </c>
       <c r="E25">
-        <v>7.0699999999999999E-2</v>
+        <v>0.28789999999999999</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>0.333486</v>
+        <v>-0.58510300000000004</v>
       </c>
       <c r="B26">
-        <v>0.55082900000000001</v>
+        <v>0.98116999999999999</v>
       </c>
       <c r="C26">
-        <v>29.512499999999999</v>
+        <v>33.8125</v>
       </c>
       <c r="D26">
-        <v>2.73</v>
+        <v>10.92</v>
       </c>
       <c r="E26">
-        <v>7.0699999999999999E-2</v>
+        <v>0.28789999999999999</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>0.33477499999999999</v>
+        <v>-0.58218800000000004</v>
       </c>
       <c r="B27">
-        <v>0.54971800000000004</v>
+        <v>0.98474899999999999</v>
       </c>
       <c r="C27">
-        <v>29.3125</v>
+        <v>33.8125</v>
       </c>
       <c r="D27">
-        <v>2.79</v>
+        <v>10.92</v>
       </c>
       <c r="E27">
-        <v>7.2300000000000003E-2</v>
+        <v>0.28789999999999999</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>0.33459100000000003</v>
+        <v>-0.57973799999999998</v>
       </c>
       <c r="B28">
-        <v>0.54960699999999996</v>
+        <v>0.98540499999999998</v>
       </c>
       <c r="C28">
-        <v>29.35</v>
+        <v>33.8125</v>
       </c>
       <c r="D28">
-        <v>2.67</v>
+        <v>10.92</v>
       </c>
       <c r="E28">
-        <v>6.9000000000000006E-2</v>
+        <v>0.28789999999999999</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>0.33459100000000003</v>
+        <v>-0.57726</v>
       </c>
       <c r="B29">
-        <v>0.54918699999999998</v>
+        <v>0.98228700000000002</v>
       </c>
       <c r="C29">
-        <v>29.35</v>
+        <v>33.825000000000003</v>
       </c>
       <c r="D29">
-        <v>2.63</v>
+        <v>10.92</v>
       </c>
       <c r="E29">
-        <v>6.8199999999999997E-2</v>
+        <v>0.28789999999999999</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30">
-        <v>0.33416099999999999</v>
+        <v>-0.57550599999999996</v>
       </c>
       <c r="B30">
-        <v>0.55045199999999994</v>
+        <v>0.98545199999999999</v>
       </c>
       <c r="C30">
-        <v>29.4</v>
+        <v>33.875</v>
       </c>
       <c r="D30">
-        <v>2.6</v>
+        <v>10.92</v>
       </c>
       <c r="E30">
-        <v>6.7400000000000002E-2</v>
+        <v>0.28789999999999999</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31">
-        <v>0.33388499999999999</v>
+        <v>-0.58247199999999999</v>
       </c>
       <c r="B31">
-        <v>0.55049599999999999</v>
+        <v>0.98438499999999995</v>
       </c>
       <c r="C31">
-        <v>29.456199999999999</v>
+        <v>33.8125</v>
       </c>
       <c r="D31">
-        <v>2.57</v>
+        <v>3.36</v>
       </c>
       <c r="E31">
-        <v>6.6600000000000006E-2</v>
+        <v>8.7499999999999994E-2</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32">
-        <v>0.33744600000000002</v>
+        <v>-0.58510300000000004</v>
       </c>
       <c r="B32">
-        <v>0.56533800000000001</v>
+        <v>0.98116999999999999</v>
       </c>
       <c r="C32">
-        <v>29.656300000000002</v>
+        <v>33.8125</v>
       </c>
       <c r="D32">
-        <v>3.04</v>
+        <v>3.36</v>
       </c>
       <c r="E32">
-        <v>7.9000000000000001E-2</v>
+        <v>8.7499999999999994E-2</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33">
-        <v>0.34392299999999998</v>
+        <v>-0.58218800000000004</v>
       </c>
       <c r="B33">
-        <v>0.56463600000000003</v>
+        <v>0.98474899999999999</v>
       </c>
       <c r="C33">
-        <v>29.324999999999999</v>
+        <v>33.8125</v>
       </c>
       <c r="D33">
-        <v>2.98</v>
+        <v>3.36</v>
       </c>
       <c r="E33">
-        <v>7.7299999999999994E-2</v>
+        <v>8.7499999999999994E-2</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34">
-        <v>0.34478300000000001</v>
+        <v>-0.57973799999999998</v>
       </c>
       <c r="B34">
-        <v>0.564272</v>
+        <v>0.98540499999999998</v>
       </c>
       <c r="C34">
-        <v>29.175000000000001</v>
+        <v>33.8125</v>
       </c>
       <c r="D34">
-        <v>2.95</v>
+        <v>3.36</v>
       </c>
       <c r="E34">
-        <v>7.6499999999999999E-2</v>
+        <v>8.7499999999999994E-2</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35">
-        <v>0.34140599999999999</v>
+        <v>-0.57726</v>
       </c>
       <c r="B35">
-        <v>0.56374899999999994</v>
+        <v>0.98228700000000002</v>
       </c>
       <c r="C35">
-        <v>29.281300000000002</v>
+        <v>33.825000000000003</v>
       </c>
       <c r="D35">
-        <v>2.95</v>
+        <v>3.36</v>
       </c>
       <c r="E35">
-        <v>7.6499999999999999E-2</v>
+        <v>8.7499999999999994E-2</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36">
-        <v>0.33938000000000001</v>
+        <v>-0.57550599999999996</v>
       </c>
       <c r="B36">
-        <v>0.56433699999999998</v>
+        <v>0.98545199999999999</v>
       </c>
       <c r="C36">
-        <v>29.462499999999999</v>
+        <v>33.875</v>
       </c>
       <c r="D36">
-        <v>2.95</v>
+        <v>3.36</v>
       </c>
       <c r="E36">
-        <v>7.6499999999999999E-2</v>
+        <v>8.7499999999999994E-2</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37">
-        <v>0.35884300000000002</v>
+        <v>-0.68544499999999997</v>
       </c>
       <c r="B37">
-        <v>0.45744200000000002</v>
+        <v>0.98711000000000004</v>
       </c>
       <c r="C37">
-        <v>26.912500000000001</v>
+        <v>34.0625</v>
       </c>
       <c r="D37">
-        <v>2.5099999999999998</v>
+        <v>3.56</v>
       </c>
       <c r="E37">
-        <v>6.5000000000000002E-2</v>
+        <v>0.92700000000000005</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38">
-        <v>0.35884300000000002</v>
+        <v>-0.68864000000000003</v>
       </c>
       <c r="B38">
-        <v>0.458144</v>
+        <v>0.981321</v>
       </c>
       <c r="C38">
-        <v>27.0063</v>
+        <v>34.0625</v>
       </c>
       <c r="D38">
-        <v>2.6</v>
+        <v>3.56</v>
       </c>
       <c r="E38">
-        <v>6.7400000000000002E-2</v>
+        <v>0.92700000000000005</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39">
-        <v>0.35675600000000002</v>
+        <v>-0.67564800000000003</v>
       </c>
       <c r="B39">
-        <v>0.459617</v>
+        <v>0.981209</v>
       </c>
       <c r="C39">
-        <v>27.1187</v>
+        <v>34.125</v>
       </c>
       <c r="D39">
-        <v>2.57</v>
+        <v>3.56</v>
       </c>
       <c r="E39">
-        <v>6.6600000000000006E-2</v>
+        <v>0.92700000000000005</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40">
-        <v>0.35509800000000002</v>
+        <v>-0.683002</v>
       </c>
       <c r="B40">
-        <v>0.45981100000000003</v>
+        <v>0.98590199999999995</v>
       </c>
       <c r="C40">
-        <v>27.237500000000001</v>
+        <v>34.125</v>
       </c>
       <c r="D40">
-        <v>2.54</v>
+        <v>3.56</v>
       </c>
       <c r="E40">
-        <v>6.5799999999999997E-2</v>
+        <v>0.92700000000000005</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41">
-        <v>0.35614200000000001</v>
+        <v>-0.69210400000000005</v>
       </c>
       <c r="B41">
-        <v>0.45699200000000001</v>
+        <v>0.98261500000000002</v>
       </c>
       <c r="C41">
-        <v>27.337499999999999</v>
+        <v>34.1875</v>
       </c>
       <c r="D41">
-        <v>2.54</v>
+        <v>3.56</v>
       </c>
       <c r="E41">
-        <v>6.5799999999999997E-2</v>
+        <v>0.92700000000000005</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42">
-        <v>0.34610299999999999</v>
+        <v>-0.68387299999999995</v>
       </c>
       <c r="B42">
-        <v>0.45958900000000003</v>
+        <v>0.98223899999999997</v>
       </c>
       <c r="C42">
-        <v>28.281300000000002</v>
+        <v>34.1875</v>
       </c>
       <c r="D42">
-        <v>3.53</v>
+        <v>3.56</v>
       </c>
       <c r="E42">
-        <v>9.1800000000000007E-2</v>
+        <v>0.92700000000000005</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43">
-        <v>0.345827</v>
+        <v>-0.54829000000000006</v>
       </c>
       <c r="B43">
-        <v>0.45967999999999998</v>
+        <v>0.98924500000000004</v>
       </c>
       <c r="C43">
-        <v>28.35</v>
+        <v>34.087499999999999</v>
       </c>
       <c r="D43">
-        <v>3.59</v>
+        <v>11.88</v>
       </c>
       <c r="E43">
-        <v>9.3600000000000003E-2</v>
+        <v>0.31319999999999998</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44">
-        <v>0.34530499999999997</v>
+        <v>-0.55379699999999998</v>
       </c>
       <c r="B44">
-        <v>0.45986500000000002</v>
+        <v>0.98223700000000003</v>
       </c>
       <c r="C44">
-        <v>28.4438</v>
+        <v>34.0625</v>
       </c>
       <c r="D44">
-        <v>3.56</v>
+        <v>11.88</v>
       </c>
       <c r="E44">
-        <v>9.2700000000000005E-2</v>
+        <v>0.31319999999999998</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45">
-        <v>0.34426099999999998</v>
+        <v>-0.54412199999999999</v>
       </c>
       <c r="B45">
-        <v>0.46132299999999998</v>
+        <v>0.98692100000000005</v>
       </c>
       <c r="C45">
-        <v>28.537500000000001</v>
+        <v>34.0625</v>
       </c>
       <c r="D45">
-        <v>3.56</v>
+        <v>11.88</v>
       </c>
       <c r="E45">
-        <v>9.2700000000000005E-2</v>
+        <v>0.31319999999999998</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46">
-        <v>0.34601100000000001</v>
+        <v>-0.54930500000000004</v>
       </c>
       <c r="B46">
-        <v>0.46150600000000003</v>
+        <v>0.98075400000000001</v>
       </c>
       <c r="C46">
-        <v>28.5063</v>
+        <v>34.075000000000003</v>
       </c>
       <c r="D46">
-        <v>3.53</v>
+        <v>11.88</v>
       </c>
       <c r="E46">
-        <v>9.1800000000000007E-2</v>
+        <v>0.31319999999999998</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47">
-        <v>0.35497499999999998</v>
+        <v>-0.546655</v>
       </c>
       <c r="B47">
-        <v>0.46775699999999998</v>
+        <v>0.98334100000000002</v>
       </c>
       <c r="C47">
-        <v>37.2562</v>
+        <v>34.125</v>
       </c>
       <c r="D47">
-        <v>4.38</v>
+        <v>11.88</v>
       </c>
       <c r="E47">
-        <v>0.1145</v>
+        <v>0.31319999999999998</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48">
-        <v>0.35537400000000002</v>
+        <v>-0.54583599999999999</v>
       </c>
       <c r="B48">
-        <v>0.46675</v>
+        <v>0.98942099999999999</v>
       </c>
       <c r="C48">
-        <v>37.412500000000001</v>
+        <v>34.125</v>
       </c>
       <c r="D48">
-        <v>4.49</v>
+        <v>11.88</v>
       </c>
       <c r="E48">
-        <v>0.1174</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A49">
-        <v>0.35571199999999997</v>
-      </c>
-      <c r="B49">
-        <v>0.46715099999999998</v>
-      </c>
-      <c r="C49">
-        <v>37.518700000000003</v>
-      </c>
-      <c r="D49">
-        <v>4.45</v>
-      </c>
-      <c r="E49">
-        <v>0.1164</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A50">
-        <v>0.35540500000000003</v>
-      </c>
-      <c r="B50">
-        <v>0.46763399999999999</v>
-      </c>
-      <c r="C50">
-        <v>37.6188</v>
-      </c>
-      <c r="D50">
-        <v>4.3099999999999996</v>
-      </c>
-      <c r="E50">
-        <v>0.11269999999999999</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A51">
-        <v>0.35644900000000002</v>
-      </c>
-      <c r="B51">
-        <v>0.46790300000000001</v>
-      </c>
-      <c r="C51">
-        <v>37.706200000000003</v>
-      </c>
-      <c r="D51">
-        <v>4.3099999999999996</v>
-      </c>
-      <c r="E51">
-        <v>0.11269999999999999</v>
+        <v>0.31319999999999998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>